<commit_message>
Use Kerala hall layout: two benches (A, B) per row; portrait seating charts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-data/exam-demo-data.xlsx
+++ b/sample-data/exam-demo-data.xlsx
@@ -6993,10 +6993,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
@@ -7009,10 +7009,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
@@ -7025,10 +7025,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>2</v>
@@ -7041,10 +7041,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
@@ -7057,10 +7057,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>
@@ -7073,10 +7073,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>

</xml_diff>